<commit_message>
modify all files for to update datas to a excel file
</commit_message>
<xml_diff>
--- a/list.xlsx
+++ b/list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsa\Desktop\code\서예\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{80E72232-6085-4FC8-BF09-82E68C3AD8B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE01027A-934A-43F9-B88A-D69CF5622CCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{2888D1DA-6869-4572-A9FC-FB1D8E207C93}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{2888D1DA-6869-4572-A9FC-FB1D8E207C93}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="53">
   <si>
     <t>작품명</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -67,6 +67,159 @@
   </si>
   <si>
     <t>‘그 나라에서 가장 뛰어난 인물은 둘도 없다.’는 뜻으로, 나라에서 견줄 사람이 없을 정도로 빼어난 선비를 말한다.</t>
+  </si>
+  <si>
+    <t>작품전 회차 (예: 제 103회)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>제 103회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>녹음방초</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>작품전 이름 (예: 녹음방초)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>작품전 한마디</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>김재원</t>
+  </si>
+  <si>
+    <t>두존쿠</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>백종현</t>
+  </si>
+  <si>
+    <t>'한 구절 위로를 구하다.'\n최근 유행했던 두쫀쿠를 발음이 비슷한 한자에 맞추어 나열했습니다.</t>
+  </si>
+  <si>
+    <t>乙瑛碑 臨書</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>손범서</t>
+  </si>
+  <si>
+    <t>靑江</t>
+  </si>
+  <si>
+    <t>을영비 임서 작품입니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>開花</t>
+  </si>
+  <si>
+    <t>신인철</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>작디작은 꽃망울이 흐르는 시간을 쫓아 만개에 이르다</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>樂天知命</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>박지현</t>
+  </si>
+  <si>
+    <t>하늘의 뜻(천명/운명)을 깨달아 즐기면서 이에 순응하고, 주어진 처지를 편안하게 받아들이는 마음가짐</t>
+  </si>
+  <si>
+    <t>벨킨 이야기, 스페이드 여왕' 발췌</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>안서영</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>알렉산드르 푸시킨의 ”벨킨이야기, 스페이드 여왕“의 문장입니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>未來</t>
+  </si>
+  <si>
+    <t>정승아</t>
+  </si>
+  <si>
+    <t>山雲</t>
+  </si>
+  <si>
+    <t>개인적으로 정말 좋아하는 단어입니다. 활기찬 미래를 향해 다들 앞으로 나가가길 바라는 마음으로 썼습니다.</t>
+  </si>
+  <si>
+    <t>里仁</t>
+  </si>
+  <si>
+    <t>변재영</t>
+  </si>
+  <si>
+    <t>淸守</t>
+  </si>
+  <si>
+    <t>최근 논어를 읽었습니다. 그 중에서도 감명 깊었던 문구를 골랐습니다. 정말 배우는 걸 좋아한다면 어디서나 배울 점을 찾아내겠죠.</t>
+  </si>
+  <si>
+    <t>言美卽響美</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>강정완</t>
+  </si>
+  <si>
+    <t>玄中</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>말이 아름다우면 울림도 아름답다.</t>
+  </si>
+  <si>
+    <t>水善利萬물而不爭</t>
+  </si>
+  <si>
+    <t>상선약수, 물은 만물을 이롭게 하되 다투지 않는다.</t>
+  </si>
+  <si>
+    <t>春興</t>
+  </si>
+  <si>
+    <t>봄의 흥취.</t>
+  </si>
+  <si>
+    <t>江南春</t>
+  </si>
+  <si>
+    <t>최민선</t>
+  </si>
+  <si>
+    <t>史香</t>
+  </si>
+  <si>
+    <t>두목의 「강남춘(江南春)」은 겉으로는 화려하고 생기 넘치는 강남의 봄 풍경을 그리지만, 과거의 번영이 이제는 안개 속처럼 희미해졌음을 표현한 시입니다.</t>
+  </si>
+  <si>
+    <t>녹음방초(綠陰芳草)에 초대합니다.</t>
+  </si>
+  <si>
+    <t>토마토</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>토마토에는 식이섬유가 풍부하다. 함유되어 있는 성분에는 구연산, 사과산, 호박산, 아미노산, 루틴, 단백질, 당질, 회분, 칼슘, 철, 인, 비타민A, 비타민 B 등이 있다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -112,8 +265,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -450,13 +606,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14CBC9D8-1A74-49C0-9749-02F03D71201F}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="4" max="4" width="100.08203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="137.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="24.08203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -469,19 +630,190 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D3" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modify  to update a date and place using the file
</commit_message>
<xml_diff>
--- a/list.xlsx
+++ b/list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsa\Desktop\code\서예\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE01027A-934A-43F9-B88A-D69CF5622CCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13CDABEB-12E7-4240-849E-A9B381007C21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{2888D1DA-6869-4572-A9FC-FB1D8E207C93}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2888D1DA-6869-4572-A9FC-FB1D8E207C93}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
   <si>
     <t>작품명</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -211,14 +211,43 @@
     <t>두목의 「강남춘(江南春)」은 겉으로는 화려하고 생기 넘치는 강남의 봄 풍경을 그리지만, 과거의 번영이 이제는 안개 속처럼 희미해졌음을 표현한 시입니다.</t>
   </si>
   <si>
+    <t>토마토</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>토마토에는 식이섬유가 풍부하다. 함유되어 있는 성분에는 구연산, 사과산, 호박산, 아미노산, 루틴, 단백질, 당질, 회분, 칼슘, 철, 인, 비타민A, 비타민 B 등이 있다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>날짜</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026.05.07 — 05.09</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>장소</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>품평회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>5월 9일</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>토요일</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>녹음방초(綠陰芳草)에 초대합니다.</t>
-  </si>
-  <si>
-    <t>토마토</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>토마토에는 식이섬유가 풍부하다. 함유되어 있는 성분에는 구연산, 사과산, 호박산, 아미노산, 루틴, 단백질, 당질, 회분, 칼슘, 철, 인, 비타민A, 비타민 B 등이 있다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>단국대학교 혜당관 2층 로비</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -265,11 +294,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -606,18 +638,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14CBC9D8-1A74-49C0-9749-02F03D71201F}">
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="45.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="4" max="4" width="137.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="24.08203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.796875" customWidth="1"/>
+    <col min="4" max="4" width="137.19921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="24.09765625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="30.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.6640625" customWidth="1"/>
+    <col min="9" max="9" width="19.59765625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -639,16 +672,25 @@
       <c r="H1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J1" t="s">
+        <v>54</v>
+      </c>
+      <c r="K1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
         <v>9</v>
@@ -657,10 +699,19 @@
         <v>10</v>
       </c>
       <c r="H2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+        <v>58</v>
+      </c>
+      <c r="I2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -673,8 +724,11 @@
       <c r="D3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="K3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -684,8 +738,11 @@
       <c r="D4" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="K4" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -699,7 +756,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -710,7 +767,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -721,7 +778,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
@@ -732,7 +789,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -746,7 +803,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -760,7 +817,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -774,7 +831,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -788,7 +845,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>44</v>
       </c>
@@ -802,7 +859,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>46</v>
       </c>

</xml_diff>